<commit_message>
progress: 39 village workbooks (rw-rtx-3070 2026-10-09T23:00:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Chitrasoor_13.392192_80.186248.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Chitrasoor_13.392192_80.186248.xlsx
@@ -710,6 +710,11 @@
           <t>276</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -717,6 +722,11 @@
           <t>277</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -724,6 +734,11 @@
           <t>278</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7A, 7B, 8, 9A1A, 9A1B, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -731,6 +746,11 @@
           <t>279</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -738,6 +758,11 @@
           <t>280</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3A, 3B, 3C, 3D, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -745,6 +770,11 @@
           <t>281</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 13, 1A, 1B, 2, 3A, 3B, 3C, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -752,6 +782,11 @@
           <t>282</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A1, 13A2, 13B, 14, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -759,6 +794,11 @@
           <t>283</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -766,6 +806,11 @@
           <t>284</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -773,6 +818,11 @@
           <t>285</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -780,6 +830,11 @@
           <t>286</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -787,6 +842,11 @@
           <t>287</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -794,6 +854,11 @@
           <t>288</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -801,6 +866,11 @@
           <t>289</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -808,6 +878,11 @@
           <t>290</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -815,6 +890,11 @@
           <t>291</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -822,6 +902,11 @@
           <t>292</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -829,6 +914,11 @@
           <t>293</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -836,6 +926,11 @@
           <t>294</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3A, 3B1, 3B2, 4A, 4B, 5A, 5B1, 5B2A, 5B2B, 5B3, 6A1, 6A2, 6B1, 6B2, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -843,6 +938,11 @@
           <t>295</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -850,6 +950,11 @@
           <t>296</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -857,6 +962,11 @@
           <t>297</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -864,6 +974,11 @@
           <t>298</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -871,6 +986,11 @@
           <t>299</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 4, 5, 6, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -878,6 +998,11 @@
           <t>300</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -885,6 +1010,11 @@
           <t>301</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -892,6 +1022,11 @@
           <t>302</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 1C, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -899,6 +1034,11 @@
           <t>303</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -906,6 +1046,11 @@
           <t>304</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -913,6 +1058,11 @@
           <t>305</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -920,6 +1070,11 @@
           <t>306</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B, 5A, 5B, 5C, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -927,6 +1082,11 @@
           <t>307</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -934,6 +1094,11 @@
           <t>308</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2A, 1B2B, 2A, 2B, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -941,6 +1106,11 @@
           <t>309</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -948,6 +1118,11 @@
           <t>310</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -955,6 +1130,11 @@
           <t>311</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -962,6 +1142,11 @@
           <t>312</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -969,6 +1154,11 @@
           <t>313</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -976,6 +1166,11 @@
           <t>314</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -983,6 +1178,11 @@
           <t>315</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -990,6 +1190,11 @@
           <t>316</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -997,6 +1202,11 @@
           <t>317</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1004,6 +1214,11 @@
           <t>318</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B1A, 1B1B, 1B2A, 1B2B, 1B3, 1B4, 1B5, 1B6, 1B7, 1B8, 1B9, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1011,6 +1226,11 @@
           <t>319</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1018,6 +1238,11 @@
           <t>320</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1025,6 +1250,11 @@
           <t>321</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1032,6 +1262,11 @@
           <t>322</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 4</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1039,6 +1274,11 @@
           <t>323</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1046,6 +1286,11 @@
           <t>324</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1053,6 +1298,11 @@
           <t>325</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1060,6 +1310,11 @@
           <t>326</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1067,6 +1322,11 @@
           <t>327</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1074,6 +1334,11 @@
           <t>328</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1081,6 +1346,11 @@
           <t>329</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1088,6 +1358,11 @@
           <t>330</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1095,6 +1370,11 @@
           <t>331</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B, 5A, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1102,6 +1382,11 @@
           <t>332</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 5C1, 5C2</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1109,6 +1394,11 @@
           <t>333</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1116,6 +1406,11 @@
           <t>334</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1123,6 +1418,11 @@
           <t>335</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1130,6 +1430,11 @@
           <t>336</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B1, 6B2</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1137,6 +1442,11 @@
           <t>337</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B1, 3B2, 4, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1144,6 +1454,11 @@
           <t>338</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1151,6 +1466,11 @@
           <t>339</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1158,6 +1478,11 @@
           <t>340</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1165,6 +1490,11 @@
           <t>341</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B1, 4B2</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1172,6 +1502,11 @@
           <t>342</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1179,6 +1514,11 @@
           <t>343</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4, 5A, 5B, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1186,6 +1526,11 @@
           <t>344</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1193,6 +1538,11 @@
           <t>345</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1200,6 +1550,11 @@
           <t>346</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 10, 11A1, 11A2, 11B1, 11B2, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1207,6 +1562,11 @@
           <t>347</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B1, 6B2</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1214,6 +1574,11 @@
           <t>348</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1221,6 +1586,11 @@
           <t>349</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3A, 3B, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1228,6 +1598,11 @@
           <t>350</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1235,6 +1610,11 @@
           <t>351</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1242,6 +1622,11 @@
           <t>352</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5A1, 5A2, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1249,6 +1634,11 @@
           <t>353</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1256,6 +1646,11 @@
           <t>354</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1263,6 +1658,11 @@
           <t>355</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1270,6 +1670,11 @@
           <t>356</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1277,6 +1682,11 @@
           <t>357</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1284,6 +1694,11 @@
           <t>358</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1291,6 +1706,11 @@
           <t>359</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1298,6 +1718,11 @@
           <t>360</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1305,6 +1730,11 @@
           <t>361</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1312,6 +1742,11 @@
           <t>362</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1, 2A, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1319,6 +1754,11 @@
           <t>363</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1326,6 +1766,11 @@
           <t>364</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1333,6 +1778,11 @@
           <t>365</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B1, 4B2, 4C1, 4C2</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1340,6 +1790,11 @@
           <t>366</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2, 2D1, 2D2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1347,6 +1802,11 @@
           <t>367</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3A, 3B, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1354,6 +1814,11 @@
           <t>368</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6A, 6B, 7A1, 7A2, 7B, 8</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1361,6 +1826,11 @@
           <t>369</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B1, 6B2</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1368,11 +1838,21 @@
           <t>370</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3, 4, 5, 6, 7A, 7B, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
           <t>371</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B1A, 4B1B, 4B2, 5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 41 village workbooks (rw-rtx-3070 2026-10-09T23:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Chitrasoor_13.392192_80.186248.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Chitrasoor_13.392192_80.186248.xlsx
@@ -1862,6 +1862,11 @@
           <t>372</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4A, 4B, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1869,11 +1874,21 @@
           <t>373</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
           <t>45</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>